<commit_message>
Add the jointcalendar and bespokeCalendar features.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_calendars.xlsx
+++ b/tests/workbooktests/workbooks/test_calendars.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9690DD57-097D-4671-A599-AB72DE620844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DBF0AE-5AA8-4EA2-90D2-68D38171C085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4560" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{93E3CEBE-2A7E-45F9-A944-9E4960940BAD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{93E3CEBE-2A7E-45F9-A944-9E4960940BAD}"/>
   </bookViews>
   <sheets>
     <sheet name="types" sheetId="1" r:id="rId1"/>
     <sheet name="functions" sheetId="2" r:id="rId2"/>
-    <sheet name="addremove holidays" sheetId="6" r:id="rId3"/>
-    <sheet name="adjust , advance" sheetId="7" r:id="rId4"/>
-    <sheet name="joined calendar" sheetId="8" r:id="rId5"/>
+    <sheet name="addremove_holidays" sheetId="6" r:id="rId3"/>
+    <sheet name="adjust_advance" sheetId="7" r:id="rId4"/>
+    <sheet name="jointCalendar" sheetId="8" r:id="rId5"/>
+    <sheet name="bespokeCalendar" sheetId="9" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="93">
   <si>
     <t>ARGENTINA</t>
   </si>
@@ -292,46 +293,58 @@
     <t>calender_rule</t>
   </si>
   <si>
+    <t>qlCalender</t>
+  </si>
+  <si>
+    <t>UK_SETTLEMENT</t>
+  </si>
+  <si>
+    <t>US_SETTLEMENT</t>
+  </si>
+  <si>
+    <t>US_FEDERALRESERVE</t>
+  </si>
+  <si>
+    <t>US_SOFR</t>
+  </si>
+  <si>
+    <t>qlCalendarJointCalendar</t>
+  </si>
+  <si>
+    <t>qlCalendarJointCalendar2</t>
+  </si>
+  <si>
+    <t>qlCalendarJointCalendar3</t>
+  </si>
+  <si>
+    <t>qlCalendarJointCalendarN</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>qlBespokeCalendar</t>
+  </si>
+  <si>
+    <t>TestCalendar</t>
+  </si>
+  <si>
+    <t>qlBespokeCalendarAddWeekend</t>
+  </si>
+  <si>
+    <t>weekday</t>
+  </si>
+  <si>
+    <t>SATURDAY</t>
+  </si>
+  <si>
+    <t>SUNDAY</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
     <t>JOINHOLIDAYS</t>
-  </si>
-  <si>
-    <t>qlCalender</t>
-  </si>
-  <si>
-    <t>UK_Settlement</t>
-  </si>
-  <si>
-    <t>UK_SETTLEMENT</t>
-  </si>
-  <si>
-    <t>US_SETTLEMENT</t>
-  </si>
-  <si>
-    <t>US_FEDERALRESERVE</t>
-  </si>
-  <si>
-    <t>US_SOFR</t>
-  </si>
-  <si>
-    <t>Denmark</t>
-  </si>
-  <si>
-    <t>Iceland</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>qlCalendarJointCalendar</t>
-  </si>
-  <si>
-    <t>qlCalendarJointCalendar2</t>
-  </si>
-  <si>
-    <t>qlCalendarJointCalendar3</t>
-  </si>
-  <si>
-    <t>qlCalendarJointCalendarN</t>
   </si>
 </sst>
 </file>
@@ -375,11 +388,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -699,6 +719,7 @@
   <cols>
     <col min="2" max="2" width="37.140625" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="33.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.25">
@@ -1090,7 +1111,7 @@
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C47" t="str">
         <f>_xll.qlCalendar(B47)</f>
@@ -1099,7 +1120,7 @@
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C48" t="str">
         <f>_xll.qlCalendar(B48)</f>
@@ -1108,7 +1129,7 @@
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C49" t="str">
         <f>_xll.qlCalendar(B49)</f>
@@ -1117,7 +1138,7 @@
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C50" t="str">
         <f>_xll.qlCalendar(B50)</f>
@@ -1136,14 +1157,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" s="4" t="str">
         <f>_xll.qlCalendar("TARGET")</f>
         <v>TARGET</v>
       </c>
@@ -1152,7 +1173,7 @@
       <c r="A2" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="5">
         <v>46171</v>
       </c>
     </row>
@@ -1160,7 +1181,7 @@
       <c r="A3" t="s">
         <v>64</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B3" s="4" t="str">
         <f>_xll.qlDateWeekday(B2)</f>
         <v>FRIDAY</v>
       </c>
@@ -1169,7 +1190,7 @@
       <c r="A4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="5">
         <v>46023</v>
       </c>
     </row>
@@ -1177,7 +1198,7 @@
       <c r="A5" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="5">
         <v>46027</v>
       </c>
       <c r="D5" s="1">
@@ -1198,7 +1219,7 @@
       <c r="A7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="b">
+      <c r="B7" s="4" t="b">
         <f>_xll.qlCalendarisWeekend($B$1,B3)</f>
         <v>0</v>
       </c>
@@ -1207,7 +1228,7 @@
       <c r="A8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="5">
         <f>_xll.qlCalendarStartOfMonth(B1,B2)</f>
         <v>46146</v>
       </c>
@@ -1216,7 +1237,7 @@
       <c r="A9" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="5">
         <f>_xll.qlCalendarEndOfMonth(B1,B2)</f>
         <v>46171</v>
       </c>
@@ -1225,7 +1246,7 @@
       <c r="A10" t="s">
         <v>46</v>
       </c>
-      <c r="B10" t="b">
+      <c r="B10" s="4" t="b">
         <f>_xll.qlCalendarIsBusinessDay(B1,B2)</f>
         <v>1</v>
       </c>
@@ -1234,7 +1255,7 @@
       <c r="A11" t="s">
         <v>47</v>
       </c>
-      <c r="B11" t="b">
+      <c r="B11" s="4" t="b">
         <f>_xll.qlCalendarIsHoliday(B1,B2)</f>
         <v>0</v>
       </c>
@@ -1243,7 +1264,7 @@
       <c r="A12" t="s">
         <v>48</v>
       </c>
-      <c r="B12" t="b">
+      <c r="B12" s="4" t="b">
         <f>_xll.qlCalendarIsEndOfMonth(B1,B2)</f>
         <v>1</v>
       </c>
@@ -1252,7 +1273,7 @@
       <c r="A13" t="s">
         <v>49</v>
       </c>
-      <c r="B13" t="b">
+      <c r="B13" s="4" t="b">
         <f>_xll.qlCalendarIsStartOfMonth(B1,B2)</f>
         <v>0</v>
       </c>
@@ -1261,7 +1282,7 @@
       <c r="A14" t="s">
         <v>53</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="4">
         <f>_xll.qlCalendarBusinessDaysBetween(B1,B4,B5)</f>
         <v>1</v>
       </c>
@@ -1270,7 +1291,7 @@
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B15" s="4" t="str">
         <f>_xll.qlCalendarName(B1)</f>
         <v>TARGET</v>
       </c>
@@ -1279,7 +1300,7 @@
       <c r="A16" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B16" t="b">
+      <c r="B16" s="4" t="b">
         <f>_xll.qlCalendarEmpty(B1)</f>
         <v>0</v>
       </c>
@@ -1288,7 +1309,7 @@
       <c r="A18" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="5">
         <f>_xll.qlCalendarHolidayList(B1,B4,B5)</f>
         <v>46023</v>
       </c>
@@ -1297,7 +1318,7 @@
       <c r="A19" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="5">
         <f>TRANSPOSE(_xll.qlCalendarBusinessDayList(B1,B4,B5))</f>
         <v>46024</v>
       </c>
@@ -1310,32 +1331,40 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41849B37-CA87-4E4A-8B76-B839138C7508}">
-  <dimension ref="A2:C18"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.42578125" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+        <v>62</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46024</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" s="1">
-        <v>46024</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B4" s="1">
         <v>46023</v>
@@ -1343,95 +1372,87 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B5" s="1">
-        <v>46023</v>
+        <v>46027</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B6" s="1">
-        <v>46027</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="1">
-        <f>_xll.qlCalendarHolidayList(B2,B5,B6,B2)</f>
+        <f>_xll.qlCalendarHolidayList(B1,B4,B5,B1)</f>
         <v>46023</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="b">
+        <f>_xll.qlCalendarAddHoliday(B1,B2,B6)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" t="b">
-        <f>_xll.qlCalendarAddHoliday(B2,B3,B7)</f>
+        <v>54</v>
+      </c>
+      <c r="B9" s="1">
+        <f>TRANSPOSE(_xll.qlCalendarHolidayList(B1,B4,B5,B8))</f>
+        <v>46023</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" t="b">
+        <f>_xll.qlCalendarRemoveHoliday(B1,B3,B9)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="1">
-        <f>TRANSPOSE(_xll.qlCalendarHolidayList(B2,B5,B6,B9))</f>
-        <v>46023</v>
-      </c>
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="1"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B12" t="b">
-        <f>_xll.qlCalendarRemoveHoliday(B2,B4,B10)</f>
+        <v>54</v>
+      </c>
+      <c r="B12" s="1">
+        <f>_xll.qlCalendarHolidayList(B1,B4,B5,B11)</f>
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="1"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" t="b">
+        <f>_xll.qlCalendarResetAddedAndRemovedHolidays(B1,B12)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="1">
-        <f>_xll.qlCalendarHolidayList(B2,B5,B6,B12)</f>
-        <v>46024</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="1"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" t="b">
-        <f>_xll.qlCalendarResetAddedAndRemovedHolidays(B2,B13)</f>
-        <v>1</v>
+        <v>54</v>
+      </c>
+      <c r="B15" s="1">
+        <f>_xll.qlCalendarHolidayList(B1,B4,B5,B14)</f>
+        <v>46023</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="1">
-        <f>_xll.qlCalendarHolidayList(B2,B5,B6,B15)</f>
-        <v>46023</v>
-      </c>
+      <c r="B16" s="1"/>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1531,7 +1552,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFBBB7C2-660D-4F66-9443-9DB0EA674324}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1539,92 +1560,212 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>84</v>
+      <c r="A1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" t="str">
+        <f>_xll.qlCalendar("Sweden")</f>
+        <v>Sweden</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" t="str">
-        <f>_xll.qlCalendar("Sweden")</f>
-        <v>Sweden</v>
+        <v>75</v>
+      </c>
+      <c r="B3" t="str" cm="1">
+        <f t="array" ref="B3">_xll.qlCalendar("UK_Settlement")</f>
+        <v>UK settlement</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+        <v>75</v>
+      </c>
+      <c r="B4" t="str" cm="1">
+        <f t="array" ref="B4">_xll.qlCalendar("Denmark")</f>
+        <v>Denmark</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" t="s">
-        <v>77</v>
+        <v>75</v>
+      </c>
+      <c r="B5" t="str" cm="1">
+        <f t="array" ref="B5">_xll.qlCalendar("Iceland")</f>
+        <v>Iceland stock exchange</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>83</v>
+      <c r="A7" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" t="str">
+        <f>_xll.qlCalendarJointCalendar(B1,B2,B6)</f>
+        <v>JoinHolidays(Sweden, TARGET)</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" t="s">
-        <v>75</v>
+      <c r="A8" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" t="str">
+        <f>_xll.qlCalendarJointCalendar2(B1,B2,B3)</f>
+        <v>JoinHolidays(Sweden, TARGET, UK settlement)</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" t="str">
-        <f>_xll.qlCalendarJointCalendar(B3,B4,B8)</f>
-        <v>JoinHolidays(Sweden, TARGET)</v>
+        <v>82</v>
+      </c>
+      <c r="B9" t="str" cm="1">
+        <f t="array" ref="B9">_xll.qlCalendarJointCalendar3(B1,B2,B3,B4,B6)</f>
+        <v>JoinHolidays(Sweden, TARGET, UK settlement, Denmark)</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B10" t="str">
-        <f>_xll.qlCalendarJointCalendar2(B3,B4,B5)</f>
-        <v>JoinHolidays(Sweden, TARGET, UK settlement)</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B11" t="str" cm="1">
-        <f t="array" ref="B11">_xll.qlCalendarJointCalendar3(B3,B4,B5,B6,B8)</f>
-        <v>JoinHolidays(Sweden, TARGET, UK settlement, Denmark)</v>
+        <v>83</v>
+      </c>
+      <c r="B10" t="str" cm="1">
+        <f t="array" ref="B10">_xll.qlCalendarJointCalendarN(B1:B5,B6)</f>
+        <v>JoinHolidays(Sweden, TARGET, UK settlement, Denmark, Iceland stock exchange)</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B12" t="str" cm="1">
-        <f t="array" ref="B12">_xll.qlCalendarJointCalendarN(B3:B7,B8)</f>
-        <v>JoinHolidays(Sweden, TARGET, UK settlement, Denmark, Iceland stock exchange)</v>
+      <c r="B12" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="4" t="b" cm="1">
+        <f t="array" ref="B13">_xll.qlCalendarisWeekend(B7,B12)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="4" t="b" cm="1">
+        <f t="array" ref="B15">_xll.qlCalendarisWeekend(B7,B14)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9414356-29FD-43C6-BF7E-7BF23ACAB286}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" t="str" cm="1">
+        <f t="array" ref="B2">_xll.qlBespokeCalendar(B1)</f>
+        <v>BESPOKECALENDAR(TestCalendar)</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="4" t="b" cm="1">
+        <f t="array" ref="B4">_xll.qlBespokeCalendarAddWeekend(B2,B3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="4" t="b" cm="1">
+        <f t="array" ref="B6">_xll.qlCalendarisWeekend(B2,B5,B4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="4" t="b" cm="1">
+        <f t="array" ref="B8">_xll.qlCalendarisWeekend(B2,B7,B6)</f>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>